<commit_message>
vault backup: 2026-09-28 17:59:57
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лабораторная работа 1.xlsx
+++ b/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лабораторная работа 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Математические методы и модели поддержки принятия решений\Лабораторные работы\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE10BE59-642D-45F6-B156-CDC8C3E360A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFEA2D2A-5D6F-4CFA-8DC7-27B42E2711FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -151,22 +151,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -457,123 +460,130 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="3" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="2">
+      <c r="B3" s="3"/>
+      <c r="C3" s="6">
+        <v>1.0000000087810401</v>
+      </c>
+      <c r="D3" s="5"/>
+    </row>
+    <row r="4" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="6">
+        <v>2.0000000087810403</v>
+      </c>
+      <c r="D4" s="5"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="6">
+        <f>3000*C3 + 4000*C4</f>
+        <v>11000.000061467283</v>
+      </c>
+      <c r="D6" s="5"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="8" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="5">
+        <v>9</v>
+      </c>
+      <c r="D8" s="5">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="5">
+        <f>5*C3 + 2 * C4</f>
+        <v>9.000000061467281</v>
+      </c>
+      <c r="D9" s="5">
+        <f>2*C3 + 4*C4</f>
+        <v>10.000000052686241</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="5">
+        <f>C4-C3</f>
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="D10" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="2">
-        <v>1.9999999999999998</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="5">
+        <f>C3</f>
+        <v>1.0000000087810401</v>
+      </c>
+      <c r="D11" s="5">
         <v>3</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="2">
-        <f>3000*C3 + 4000*C4</f>
-        <v>11000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4"/>
-    </row>
-    <row r="8" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="1">
-        <v>9</v>
-      </c>
-      <c r="D8" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="1">
-        <f>5*C3 + 2 * C4</f>
-        <v>9</v>
-      </c>
-      <c r="D9" s="1">
-        <f>2*C3 + 4*C4</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="1">
-        <f>C4-C3</f>
-        <v>0.99999999999999978</v>
-      </c>
-      <c r="D10" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="1">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="5">
         <f>C3</f>
-        <v>1</v>
-      </c>
-      <c r="D11" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="1">
-        <f>C3</f>
-        <v>1</v>
-      </c>
-      <c r="D12" s="1">
+        <v>1.0000000087810401</v>
+      </c>
+      <c r="D12" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="1">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="5">
         <f>C4</f>
-        <v>1.9999999999999998</v>
-      </c>
-      <c r="D13" s="1">
+        <v>2.0000000087810403</v>
+      </c>
+      <c r="D13" s="5">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-28 18:04:38
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лабораторная работа 1.xlsx
+++ b/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лабораторная работа 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Математические методы и модели поддержки принятия решений\Лабораторные работы\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFEA2D2A-5D6F-4CFA-8DC7-27B42E2711FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDA3202-9CA2-4982-9788-8C931786E35A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -159,17 +159,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -460,81 +460,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
     </row>
     <row r="3" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="6">
+      <c r="B3" s="5"/>
+      <c r="C3" s="4">
         <v>1.0000000087810401</v>
       </c>
-      <c r="D3" s="5"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="6">
+      <c r="B4" s="5"/>
+      <c r="C4" s="4">
         <v>2.0000000087810403</v>
       </c>
-      <c r="D4" s="5"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="6">
+      <c r="B6" s="5"/>
+      <c r="C6" s="4">
         <f>3000*C3 + 4000*C4</f>
         <v>11000.000061467283</v>
       </c>
-      <c r="D6" s="5"/>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
     </row>
     <row r="8" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="5">
+      <c r="B8" s="5"/>
+      <c r="C8" s="3">
         <v>9</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="3">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
-      <c r="C9" s="5">
+      <c r="C9" s="3">
         <f>5*C3 + 2 * C4</f>
         <v>9.000000061467281</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="3">
         <f>2*C3 + 4*C4</f>
         <v>10.000000052686241</v>
       </c>
@@ -544,22 +544,22 @@
       <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="3">
         <f>C4-C3</f>
         <v>1.0000000000000002</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
-      <c r="C11" s="5">
+      <c r="C11" s="3">
         <f>C3</f>
         <v>1.0000000087810401</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="3">
         <v>3</v>
       </c>
     </row>
@@ -568,22 +568,22 @@
       <c r="B12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="3">
         <f>C3</f>
         <v>1.0000000087810401</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
-      <c r="C13" s="5">
+      <c r="C13" s="3">
         <f>C4</f>
         <v>2.0000000087810403</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-28 18:06:24
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лабораторная работа 1.xlsx
+++ b/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лабораторная работа 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Математические методы и модели поддержки принятия решений\Лабораторные работы\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDA3202-9CA2-4982-9788-8C931786E35A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCA23358-FE90-4B93-872B-BCC5EC14B647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,8 +26,8 @@
     <definedName name="solver_lhs2" localSheetId="0" hidden="1">Лист2!$C$11</definedName>
     <definedName name="solver_lhs3" localSheetId="0" hidden="1">Лист2!$C$12</definedName>
     <definedName name="solver_lhs4" localSheetId="0" hidden="1">Лист2!$C$13</definedName>
-    <definedName name="solver_lhs5" localSheetId="0" hidden="1">Лист2!$C$9</definedName>
-    <definedName name="solver_lhs6" localSheetId="0" hidden="1">Лист2!$D$9</definedName>
+    <definedName name="solver_lhs5" localSheetId="0" hidden="1">Лист2!$C$8</definedName>
+    <definedName name="solver_lhs6" localSheetId="0" hidden="1">Лист2!$C$9</definedName>
     <definedName name="solver_mip" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_mni" localSheetId="0" hidden="1">30</definedName>
     <definedName name="solver_mrt" localSheetId="0" hidden="1">0.075</definedName>
@@ -49,8 +49,8 @@
     <definedName name="solver_rhs2" localSheetId="0" hidden="1">Лист2!$D$11</definedName>
     <definedName name="solver_rhs3" localSheetId="0" hidden="1">Лист2!$D$12</definedName>
     <definedName name="solver_rhs4" localSheetId="0" hidden="1">Лист2!$D$13</definedName>
-    <definedName name="solver_rhs5" localSheetId="0" hidden="1">Лист2!$C$8</definedName>
-    <definedName name="solver_rhs6" localSheetId="0" hidden="1">Лист2!$D$8</definedName>
+    <definedName name="solver_rhs5" localSheetId="0" hidden="1">Лист2!$D$8</definedName>
+    <definedName name="solver_rhs6" localSheetId="0" hidden="1">Лист2!$D$9</definedName>
     <definedName name="solver_rlx" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rsd" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_scl" localSheetId="0" hidden="1">1</definedName>
@@ -113,6 +113,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -159,17 +162,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -460,83 +463,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="3" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="4">
+      <c r="B3" s="3"/>
+      <c r="C3" s="5">
         <v>1.0000000087810401</v>
       </c>
-      <c r="D3" s="3"/>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="4">
+      <c r="B4" s="3"/>
+      <c r="C4" s="5">
         <v>2.0000000087810403</v>
       </c>
-      <c r="D4" s="3"/>
+      <c r="D4" s="6"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="4">
+      <c r="B6" s="3"/>
+      <c r="C6" s="5">
         <f>3000*C3 + 4000*C4</f>
         <v>11000.000061467283</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="6"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
     </row>
     <row r="8" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="3">
-        <v>9</v>
-      </c>
-      <c r="D8" s="3">
+      <c r="B8" s="3"/>
+      <c r="C8" s="6">
+        <f>2*$C$3 + 4*$C$4</f>
+        <v>10.000000052686241</v>
+      </c>
+      <c r="D8" s="6">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
-      <c r="C9" s="3">
+      <c r="C9" s="6">
         <f>5*C3 + 2 * C4</f>
         <v>9.000000061467281</v>
       </c>
-      <c r="D9" s="3">
-        <f>2*C3 + 4*C4</f>
-        <v>10.000000052686241</v>
+      <c r="D9" s="6">
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -544,22 +547,22 @@
       <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="6">
         <f>C4-C3</f>
         <v>1.0000000000000002</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
-      <c r="C11" s="3">
+      <c r="C11" s="6">
         <f>C3</f>
         <v>1.0000000087810401</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="6">
         <v>3</v>
       </c>
     </row>
@@ -568,22 +571,22 @@
       <c r="B12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="6">
         <f>C3</f>
         <v>1.0000000087810401</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
-      <c r="C13" s="3">
+      <c r="C13" s="6">
         <f>C4</f>
         <v>2.0000000087810403</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="6">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-28 18:18:14
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лабораторная работа 1.xlsx
+++ b/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лабораторная работа 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Математические методы и модели поддержки принятия решений\Лабораторные работы\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCA23358-FE90-4B93-872B-BCC5EC14B647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25E60D6D-862C-4A37-8764-D08C928A645B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист2" sheetId="2" r:id="rId1"/>
@@ -479,7 +479,7 @@
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="5">
-        <v>1.0000000087810401</v>
+        <v>1</v>
       </c>
       <c r="D3" s="6"/>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="5">
-        <v>2.0000000087810403</v>
+        <v>1.9999999999999998</v>
       </c>
       <c r="D4" s="6"/>
     </row>
@@ -506,7 +506,7 @@
       <c r="B6" s="3"/>
       <c r="C6" s="5">
         <f>3000*C3 + 4000*C4</f>
-        <v>11000.000061467283</v>
+        <v>11000</v>
       </c>
       <c r="D6" s="6"/>
     </row>
@@ -525,7 +525,7 @@
       <c r="B8" s="3"/>
       <c r="C8" s="6">
         <f>2*$C$3 + 4*$C$4</f>
-        <v>10.000000052686241</v>
+        <v>10</v>
       </c>
       <c r="D8" s="6">
         <v>12</v>
@@ -536,7 +536,7 @@
       <c r="B9" s="2"/>
       <c r="C9" s="6">
         <f>5*C3 + 2 * C4</f>
-        <v>9.000000061467281</v>
+        <v>9</v>
       </c>
       <c r="D9" s="6">
         <v>9</v>
@@ -549,7 +549,7 @@
       </c>
       <c r="C10" s="6">
         <f>C4-C3</f>
-        <v>1.0000000000000002</v>
+        <v>0.99999999999999978</v>
       </c>
       <c r="D10" s="6">
         <v>1</v>
@@ -560,7 +560,7 @@
       <c r="B11" s="2"/>
       <c r="C11" s="6">
         <f>C3</f>
-        <v>1.0000000087810401</v>
+        <v>1</v>
       </c>
       <c r="D11" s="6">
         <v>3</v>
@@ -573,7 +573,7 @@
       </c>
       <c r="C12" s="6">
         <f>C3</f>
-        <v>1.0000000087810401</v>
+        <v>1</v>
       </c>
       <c r="D12" s="6">
         <v>0</v>
@@ -584,7 +584,7 @@
       <c r="B13" s="2"/>
       <c r="C13" s="6">
         <f>C4</f>
-        <v>2.0000000087810403</v>
+        <v>1.9999999999999998</v>
       </c>
       <c r="D13" s="6">
         <v>0</v>

</xml_diff>